<commit_message>
BRD-02 v2.1: FRS and UX screen documents rebuilt on the retaken document images
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-1_Transactional/BRD-02_Operations/08_BIBS_UXScreens_BRD-02_Operations_v2.1.xlsx
+++ b/docs/deliverables/out/Drop-1_Transactional/BRD-02_Operations/08_BIBS_UXScreens_BRD-02_Operations_v2.1.xlsx
@@ -11609,7 +11609,7 @@
       </c>
       <c r="K167" s="45" t="inlineStr">
         <is>
-          <t>Production register: first page as generated</t>
+          <t>Production register: first page as generated, with a selection of the columns</t>
         </is>
       </c>
       <c r="L167" s="45" t="inlineStr">
@@ -11669,7 +11669,7 @@
       </c>
       <c r="K168" s="45" t="inlineStr">
         <is>
-          <t>Direct payment commission billing: first page as generated</t>
+          <t>Direct payment commission billing: first page as generated, with a selection of the columns</t>
         </is>
       </c>
       <c r="L168" s="45" t="inlineStr">

</xml_diff>